<commit_message>
added updates to template - blocked, pass %, fail%
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="102">
   <si>
     <t>Weekly SIT Status Report</t>
   </si>
@@ -113,6 +113,9 @@
     <t>Failed</t>
   </si>
   <si>
+    <t>Blocked</t>
+  </si>
+  <si>
     <t>Pass %</t>
   </si>
   <si>
@@ -254,10 +257,10 @@
     <t xml:space="preserve">  1. Select A1:H5 (headers + 4 workstream rows)</t>
   </si>
   <si>
-    <t xml:space="preserve">  2. Insert → Charts → Clustered Bar (shows Planned/Executed/Passed/Failed side by side)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  3. Or select A1:A5 + H1:H5 for a Pass Rate bar chart per workstream</t>
+    <t xml:space="preserve">  2. Insert → Charts → Clustered Bar (shows Planned/Executed/Passed/Failed/Blocked side by side)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  3. Or select A1:A5 + I1:I5 for a Pass Rate bar chart per workstream</t>
   </si>
   <si>
     <t>Sheet "Sub-Suites":</t>
@@ -377,7 +380,7 @@
       <name val="Courier New"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -409,6 +412,11 @@
         <fgColor rgb="FFE0E7FF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEF3C7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -437,7 +445,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -483,6 +491,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -998,16 +1009,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="5" width="12" customWidth="1"/>
     <col min="6" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="8" max="9" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>27</v>
       </c>
@@ -1032,10 +1043,13 @@
       <c r="H1" s="5" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B2" s="16">
         <v>120</v>
@@ -1050,23 +1064,26 @@
         <v>15</v>
       </c>
       <c r="F2" s="16">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="G2" s="16">
         <v>0</v>
       </c>
-      <c r="H2" s="17" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H2" s="19">
+        <v>5</v>
+      </c>
+      <c r="I2" s="17" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="B3" s="19">
+        <v>36</v>
+      </c>
+      <c r="B3" s="20">
         <v>85</v>
       </c>
-      <c r="C3" s="19">
+      <c r="C3" s="20">
         <v>70</v>
       </c>
       <c r="D3" s="17">
@@ -1075,19 +1092,22 @@
       <c r="E3" s="18">
         <v>5</v>
       </c>
-      <c r="F3" s="19">
+      <c r="F3" s="20">
         <v>15</v>
       </c>
-      <c r="G3" s="19">
+      <c r="G3" s="20">
         <v>0</v>
       </c>
-      <c r="H3" s="17" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H3" s="20">
+        <v>0</v>
+      </c>
+      <c r="I3" s="17" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B4" s="16">
         <v>100</v>
@@ -1107,18 +1127,21 @@
       <c r="G4" s="16">
         <v>0</v>
       </c>
-      <c r="H4" s="17" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H4" s="16">
+        <v>0</v>
+      </c>
+      <c r="I4" s="17" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B5" s="19">
+        <v>40</v>
+      </c>
+      <c r="B5" s="20">
         <v>60</v>
       </c>
-      <c r="C5" s="19">
+      <c r="C5" s="20">
         <v>45</v>
       </c>
       <c r="D5" s="17">
@@ -1127,45 +1150,51 @@
       <c r="E5" s="18">
         <v>5</v>
       </c>
-      <c r="F5" s="19">
-        <v>15</v>
-      </c>
-      <c r="G5" s="19">
+      <c r="F5" s="20">
+        <v>13</v>
+      </c>
+      <c r="G5" s="20">
         <v>0</v>
       </c>
-      <c r="H5" s="17" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="20" t="s">
+      <c r="H5" s="19">
+        <v>2</v>
+      </c>
+      <c r="I5" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="B6" s="21">
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="21" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="22">
         <v>365</v>
       </c>
-      <c r="C6" s="21">
+      <c r="C6" s="22">
         <v>298</v>
       </c>
-      <c r="D6" s="21">
+      <c r="D6" s="22">
         <v>260</v>
       </c>
-      <c r="E6" s="21">
+      <c r="E6" s="22">
         <v>38</v>
       </c>
-      <c r="F6" s="21">
-        <v>67</v>
-      </c>
-      <c r="G6" s="21">
+      <c r="F6" s="22">
+        <v>60</v>
+      </c>
+      <c r="G6" s="22">
         <v>0</v>
       </c>
-      <c r="H6" s="22" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H6" s="22">
+        <v>7</v>
+      </c>
+      <c r="I6" s="23" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="15" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
@@ -1174,11 +1203,12 @@
       <c r="F8" s="15"/>
       <c r="G8" s="15"/>
       <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1"/>
+  <autoFilter ref="A1:I1"/>
   <mergeCells count="1">
-    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A8:I8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1187,18 +1217,18 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="5" width="12" customWidth="1"/>
     <col min="6" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="8" max="9" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>28</v>
@@ -1221,22 +1251,26 @@
       <c r="H1" s="5" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="23" t="s">
+      <c r="I1" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
+      <c r="I2" s="24"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B3" s="16">
         <v>120</v>
@@ -1251,23 +1285,26 @@
         <v>15</v>
       </c>
       <c r="F3" s="16">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="G3" s="16">
         <v>0</v>
       </c>
-      <c r="H3" s="17" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H3" s="19">
+        <v>5</v>
+      </c>
+      <c r="I3" s="17" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="B4" s="19">
+        <v>47</v>
+      </c>
+      <c r="B4" s="20">
         <v>60</v>
       </c>
-      <c r="C4" s="19">
+      <c r="C4" s="20">
         <v>48</v>
       </c>
       <c r="D4" s="17">
@@ -1276,19 +1313,22 @@
       <c r="E4" s="18">
         <v>6</v>
       </c>
-      <c r="F4" s="19">
-        <v>12</v>
-      </c>
-      <c r="G4" s="19">
+      <c r="F4" s="20">
+        <v>10</v>
+      </c>
+      <c r="G4" s="20">
         <v>0</v>
       </c>
-      <c r="H4" s="17" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H4" s="19">
+        <v>2</v>
+      </c>
+      <c r="I4" s="17" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B5" s="16">
         <v>30</v>
@@ -1303,23 +1343,26 @@
         <v>2</v>
       </c>
       <c r="F5" s="16">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G5" s="16">
         <v>0</v>
       </c>
-      <c r="H5" s="17" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H5" s="19">
+        <v>1</v>
+      </c>
+      <c r="I5" s="17" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="B6" s="19">
+        <v>51</v>
+      </c>
+      <c r="B6" s="20">
         <v>15</v>
       </c>
-      <c r="C6" s="19">
+      <c r="C6" s="20">
         <v>12</v>
       </c>
       <c r="D6" s="17">
@@ -1328,19 +1371,22 @@
       <c r="E6" s="18">
         <v>1</v>
       </c>
-      <c r="F6" s="19">
-        <v>3</v>
-      </c>
-      <c r="G6" s="19">
+      <c r="F6" s="20">
+        <v>2</v>
+      </c>
+      <c r="G6" s="20">
         <v>0</v>
       </c>
-      <c r="H6" s="17" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H6" s="19">
+        <v>1</v>
+      </c>
+      <c r="I6" s="17" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="15" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
@@ -1349,12 +1395,13 @@
       <c r="F8" s="15"/>
       <c r="G8" s="15"/>
       <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1"/>
+  <autoFilter ref="A1:I1"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A8:I8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1371,154 +1418,154 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
-        <v>52</v>
-      </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
+      <c r="A1" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B3" s="16">
         <v>3</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="B4" s="19">
+        <v>58</v>
+      </c>
+      <c r="B4" s="20">
         <v>12</v>
       </c>
-      <c r="C4" s="19" t="s">
-        <v>58</v>
+      <c r="C4" s="20" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B5" s="16">
         <v>18</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="B6" s="19">
+        <v>62</v>
+      </c>
+      <c r="B6" s="20">
         <v>4</v>
       </c>
-      <c r="C6" s="19" t="s">
-        <v>62</v>
+      <c r="C6" s="20" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="24" t="s">
-        <v>41</v>
-      </c>
-      <c r="B7" s="25">
+      <c r="A7" s="25" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" s="26">
         <v>37</v>
       </c>
-      <c r="C7" s="25" t="s">
-        <v>63</v>
+      <c r="C7" s="26" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="23" t="s">
-        <v>64</v>
-      </c>
-      <c r="B9" s="23"/>
-      <c r="C9" s="23"/>
+      <c r="A9" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="B9" s="24"/>
+      <c r="C9" s="24"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>9</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B11" s="16">
         <v>5</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="B12" s="19">
+        <v>68</v>
+      </c>
+      <c r="B12" s="20">
         <v>15</v>
       </c>
-      <c r="C12" s="19" t="s">
-        <v>68</v>
+      <c r="C12" s="20" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B13" s="16">
         <v>12</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="B14" s="19">
+        <v>71</v>
+      </c>
+      <c r="B14" s="20">
         <v>5</v>
       </c>
-      <c r="C14" s="19" t="s">
-        <v>71</v>
+      <c r="C14" s="20" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="24" t="s">
-        <v>41</v>
-      </c>
-      <c r="B15" s="25">
+      <c r="A15" s="25" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15" s="26">
         <v>37</v>
       </c>
-      <c r="C15" s="25" t="s">
-        <v>63</v>
+      <c r="C15" s="26" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B17" s="15"/>
       <c r="C17" s="15"/>
@@ -1543,183 +1590,183 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="26" t="s">
-        <v>73</v>
+      <c r="A1" s="27" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
-        <v>74</v>
+      <c r="A2" s="28" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="28" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" s="28" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="27" t="s">
-        <v>74</v>
-      </c>
-    </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="28" t="s">
-        <v>76</v>
+      <c r="A5" s="29" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="27" t="s">
-        <v>74</v>
+      <c r="A6" s="28" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="27" t="s">
-        <v>77</v>
+      <c r="A7" s="28" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="27" t="s">
-        <v>78</v>
+      <c r="A8" s="28" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="27" t="s">
-        <v>79</v>
+      <c r="A9" s="28" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="27" t="s">
-        <v>80</v>
+      <c r="A10" s="28" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="27" t="s">
-        <v>74</v>
+      <c r="A11" s="28" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="27" t="s">
-        <v>81</v>
+      <c r="A12" s="28" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="27" t="s">
-        <v>82</v>
+      <c r="A13" s="28" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" s="27" t="s">
-        <v>83</v>
+      <c r="A14" s="28" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="27" t="s">
-        <v>74</v>
+      <c r="A15" s="28" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" s="27" t="s">
-        <v>84</v>
+      <c r="A16" s="28" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="27" t="s">
-        <v>85</v>
+      <c r="A17" s="28" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="27" t="s">
-        <v>86</v>
+      <c r="A18" s="28" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="27" t="s">
-        <v>74</v>
+      <c r="A19" s="28" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" s="28" t="s">
-        <v>87</v>
+      <c r="A20" s="29" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" s="27" t="s">
-        <v>74</v>
+      <c r="A21" s="28" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" s="29" t="s">
-        <v>88</v>
+      <c r="A22" s="30" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" s="29" t="s">
-        <v>89</v>
+      <c r="A23" s="30" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" s="29" t="s">
-        <v>90</v>
+      <c r="A24" s="30" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" s="29" t="s">
-        <v>91</v>
+      <c r="A25" s="30" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" s="29" t="s">
-        <v>92</v>
+      <c r="A26" s="30" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A27" s="29" t="s">
-        <v>93</v>
+      <c r="A27" s="30" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A28" s="29" t="s">
-        <v>94</v>
+      <c r="A28" s="30" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A29" s="29" t="s">
-        <v>95</v>
+      <c r="A29" s="30" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A30" s="29" t="s">
-        <v>96</v>
+      <c r="A30" s="30" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A31" s="29" t="s">
-        <v>97</v>
+      <c r="A31" s="30" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A32" s="29" t="s">
-        <v>98</v>
+      <c r="A32" s="30" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33" s="27" t="s">
-        <v>74</v>
+      <c r="A33" s="28" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34" s="27" t="s">
-        <v>99</v>
+      <c r="A34" s="28" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A35" s="27" t="s">
-        <v>74</v>
+      <c r="A35" s="28" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A36" s="27" t="s">
-        <v>100</v>
+      <c r="A36" s="28" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>